<commit_message>
REFACTORIZACION DE INTERFAZ Y NUEVAS MODALIDADES
</commit_message>
<xml_diff>
--- a/BACKEND/marcajes.xlsx
+++ b/BACKEND/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="120">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -338,6 +338,39 @@
   </si>
   <si>
     <t>09/09/2026, 10:10:43 a. m.</t>
+  </si>
+  <si>
+    <t>10/09/2026, 10:46:36 a. m.</t>
+  </si>
+  <si>
+    <t>10/09/2026, 06:21:17 p. m.</t>
+  </si>
+  <si>
+    <t>11/09/2026, 01:46:40 p. m.</t>
+  </si>
+  <si>
+    <t>11/09/2026, 03:04:36 p. m.</t>
+  </si>
+  <si>
+    <t>12/09/2026, 10:08:04 a. m.</t>
+  </si>
+  <si>
+    <t>12/09/2026, 11:21:20 a. m.</t>
+  </si>
+  <si>
+    <t>EMANUEL DAVID APONTE MARCANO</t>
+  </si>
+  <si>
+    <t>12/09/2026, 04:27:23 p. m.</t>
+  </si>
+  <si>
+    <t>JONATHAN JOSE FARIAS RODRIGUEZ</t>
+  </si>
+  <si>
+    <t>13/09/2026, 08:09:01 a. m.</t>
+  </si>
+  <si>
+    <t>13/09/2026, 08:28:51 a. m.</t>
   </si>
 </sst>
 </file>
@@ -726,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2249,6 +2282,159 @@
         <v>9</v>
       </c>
     </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>71</v>
+      </c>
+      <c r="B90" t="s">
+        <v>72</v>
+      </c>
+      <c r="C90" t="s">
+        <v>109</v>
+      </c>
+      <c r="D90" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>17</v>
+      </c>
+      <c r="B91" t="s">
+        <v>18</v>
+      </c>
+      <c r="C91" t="s">
+        <v>110</v>
+      </c>
+      <c r="D91" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>17</v>
+      </c>
+      <c r="B92" t="s">
+        <v>18</v>
+      </c>
+      <c r="C92" t="s">
+        <v>111</v>
+      </c>
+      <c r="D92" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>17</v>
+      </c>
+      <c r="B93" t="s">
+        <v>18</v>
+      </c>
+      <c r="C93" t="s">
+        <v>112</v>
+      </c>
+      <c r="D93" t="s">
+        <v>8</v>
+      </c>
+      <c r="E93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>71</v>
+      </c>
+      <c r="B94" t="s">
+        <v>72</v>
+      </c>
+      <c r="C94" t="s">
+        <v>113</v>
+      </c>
+      <c r="D94" t="s">
+        <v>8</v>
+      </c>
+      <c r="E94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>5</v>
+      </c>
+      <c r="B95" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" t="s">
+        <v>114</v>
+      </c>
+      <c r="D95" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>17</v>
+      </c>
+      <c r="B96" t="s">
+        <v>115</v>
+      </c>
+      <c r="C96" t="s">
+        <v>116</v>
+      </c>
+      <c r="D96" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>5</v>
+      </c>
+      <c r="B97" t="s">
+        <v>117</v>
+      </c>
+      <c r="C97" t="s">
+        <v>118</v>
+      </c>
+      <c r="D97" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>17</v>
+      </c>
+      <c r="B98" t="s">
+        <v>115</v>
+      </c>
+      <c r="C98" t="s">
+        <v>119</v>
+      </c>
+      <c r="D98" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
interfaz finalizada multiplataforma - voy a refactorizar backend ahora
</commit_message>
<xml_diff>
--- a/BACKEND/marcajes.xlsx
+++ b/BACKEND/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="126">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -371,6 +371,24 @@
   </si>
   <si>
     <t>13/09/2026, 08:28:51 a. m.</t>
+  </si>
+  <si>
+    <t>13/09/2026, 07:16:17 p. m.</t>
+  </si>
+  <si>
+    <t>14/09/2026, 07:46:46 p. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:01:25 a. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:25:07 a. m.</t>
+  </si>
+  <si>
+    <t>LUIS JOSE ROJAS MONTERO</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:28:03 a. m.</t>
   </si>
 </sst>
 </file>
@@ -759,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2435,6 +2453,91 @@
         <v>9</v>
       </c>
     </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>5</v>
+      </c>
+      <c r="B99" t="s">
+        <v>117</v>
+      </c>
+      <c r="C99" t="s">
+        <v>120</v>
+      </c>
+      <c r="D99" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>5</v>
+      </c>
+      <c r="B100" t="s">
+        <v>117</v>
+      </c>
+      <c r="C100" t="s">
+        <v>121</v>
+      </c>
+      <c r="D100" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>17</v>
+      </c>
+      <c r="B101" t="s">
+        <v>115</v>
+      </c>
+      <c r="C101" t="s">
+        <v>122</v>
+      </c>
+      <c r="D101" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>82</v>
+      </c>
+      <c r="B102" t="s">
+        <v>83</v>
+      </c>
+      <c r="C102" t="s">
+        <v>123</v>
+      </c>
+      <c r="D102" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>71</v>
+      </c>
+      <c r="B103" t="s">
+        <v>124</v>
+      </c>
+      <c r="C103" t="s">
+        <v>125</v>
+      </c>
+      <c r="D103" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
refactor: fusion exitosa de codigo biometrico y mejoras en master
</commit_message>
<xml_diff>
--- a/BACKEND/marcajes.xlsx
+++ b/BACKEND/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="133">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -31,7 +31,7 @@
     <t>27280588</t>
   </si>
   <si>
-    <t>JONATHAN FARIAS</t>
+    <t>JONATHAN JOSE FARIAS RODRIGUEZ</t>
   </si>
   <si>
     <t>23/08/2026, 01:19:05 p. m.</t>
@@ -67,7 +67,7 @@
     <t>29789773</t>
   </si>
   <si>
-    <t>EMANUEL APONTE</t>
+    <t>EMANUEL DAVID APONTE MARCANO</t>
   </si>
   <si>
     <t>23/08/2026, 01:55:44 p. m.</t>
@@ -229,7 +229,7 @@
     <t>24765865</t>
   </si>
   <si>
-    <t>LUIS ROJAS</t>
+    <t>LUIS JOSE ROJAS MONTERO</t>
   </si>
   <si>
     <t>29/08/2026, 02:06:46 p. m.</t>
@@ -358,19 +358,58 @@
     <t>12/09/2026, 11:21:20 a. m.</t>
   </si>
   <si>
-    <t>EMANUEL DAVID APONTE MARCANO</t>
-  </si>
-  <si>
     <t>12/09/2026, 04:27:23 p. m.</t>
   </si>
   <si>
-    <t>JONATHAN JOSE FARIAS RODRIGUEZ</t>
-  </si>
-  <si>
     <t>13/09/2026, 08:09:01 a. m.</t>
   </si>
   <si>
     <t>13/09/2026, 08:28:51 a. m.</t>
+  </si>
+  <si>
+    <t>13/09/2026, 07:16:17 p. m.</t>
+  </si>
+  <si>
+    <t>14/09/2026, 07:46:46 p. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:01:25 a. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:25:07 a. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 10:28:03 a. m.</t>
+  </si>
+  <si>
+    <t>15/09/2026, 07:57:28 p. m.</t>
+  </si>
+  <si>
+    <t>16/09/2026, 07:54:26 a. m.</t>
+  </si>
+  <si>
+    <t>16/09/2026, 07:54:35 a. m.</t>
+  </si>
+  <si>
+    <t>16/09/2026, 08:04:17 a. m.</t>
+  </si>
+  <si>
+    <t>26082578</t>
+  </si>
+  <si>
+    <t>ALEXIS ZABALA</t>
+  </si>
+  <si>
+    <t>16/09/2026, 08:05:39 a. m.</t>
+  </si>
+  <si>
+    <t>29591045</t>
+  </si>
+  <si>
+    <t>ADRIANA SUBERO</t>
+  </si>
+  <si>
+    <t>16/09/2026, 08:07:09 a. m.</t>
   </si>
 </sst>
 </file>
@@ -759,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2389,10 +2428,10 @@
         <v>17</v>
       </c>
       <c r="B96" t="s">
+        <v>18</v>
+      </c>
+      <c r="C96" t="s">
         <v>115</v>
-      </c>
-      <c r="C96" t="s">
-        <v>116</v>
       </c>
       <c r="D96" t="s">
         <v>8</v>
@@ -2406,10 +2445,10 @@
         <v>5</v>
       </c>
       <c r="B97" t="s">
-        <v>117</v>
+        <v>6</v>
       </c>
       <c r="C97" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D97" t="s">
         <v>8</v>
@@ -2423,15 +2462,202 @@
         <v>17</v>
       </c>
       <c r="B98" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="C98" t="s">
+        <v>117</v>
+      </c>
+      <c r="D98" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>5</v>
+      </c>
+      <c r="B99" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" t="s">
+        <v>118</v>
+      </c>
+      <c r="D99" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>5</v>
+      </c>
+      <c r="B100" t="s">
+        <v>6</v>
+      </c>
+      <c r="C100" t="s">
         <v>119</v>
       </c>
-      <c r="D98" t="s">
-        <v>8</v>
-      </c>
-      <c r="E98" t="s">
+      <c r="D100" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>17</v>
+      </c>
+      <c r="B101" t="s">
+        <v>18</v>
+      </c>
+      <c r="C101" t="s">
+        <v>120</v>
+      </c>
+      <c r="D101" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>82</v>
+      </c>
+      <c r="B102" t="s">
+        <v>83</v>
+      </c>
+      <c r="C102" t="s">
+        <v>121</v>
+      </c>
+      <c r="D102" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>71</v>
+      </c>
+      <c r="B103" t="s">
+        <v>72</v>
+      </c>
+      <c r="C103" t="s">
+        <v>122</v>
+      </c>
+      <c r="D103" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>17</v>
+      </c>
+      <c r="B104" t="s">
+        <v>18</v>
+      </c>
+      <c r="C104" t="s">
+        <v>123</v>
+      </c>
+      <c r="D104" t="s">
+        <v>8</v>
+      </c>
+      <c r="E104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>82</v>
+      </c>
+      <c r="B105" t="s">
+        <v>83</v>
+      </c>
+      <c r="C105" t="s">
+        <v>124</v>
+      </c>
+      <c r="D105" t="s">
+        <v>8</v>
+      </c>
+      <c r="E105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>5</v>
+      </c>
+      <c r="B106" t="s">
+        <v>6</v>
+      </c>
+      <c r="C106" t="s">
+        <v>125</v>
+      </c>
+      <c r="D106" t="s">
+        <v>8</v>
+      </c>
+      <c r="E106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>71</v>
+      </c>
+      <c r="B107" t="s">
+        <v>72</v>
+      </c>
+      <c r="C107" t="s">
+        <v>126</v>
+      </c>
+      <c r="D107" t="s">
+        <v>8</v>
+      </c>
+      <c r="E107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>127</v>
+      </c>
+      <c r="B108" t="s">
+        <v>128</v>
+      </c>
+      <c r="C108" t="s">
+        <v>129</v>
+      </c>
+      <c r="D108" t="s">
+        <v>8</v>
+      </c>
+      <c r="E108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>130</v>
+      </c>
+      <c r="B109" t="s">
+        <v>131</v>
+      </c>
+      <c r="C109" t="s">
+        <v>132</v>
+      </c>
+      <c r="D109" t="s">
+        <v>8</v>
+      </c>
+      <c r="E109" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>